<commit_message>
QA follow-ups: LG TOC pages, cover version, formula wrap, Lab 3 source totals
- inject_toc: match a heading where it starts a line, so the topic lead-in
  that lists concept names no longer steals the page (18 LG entries fixed).
- Deck cover: version line moved under the title, off the orange circle.
- Lab PDFs: long formula lines shrink to fit one line instead of wrapping
  mid-token (Lab 3 Step 3 SUMIFS copied broken).
- Lab 3 data: tblSources applications/hires now add up to tblMonthly's
  2026 totals (6,616 / 361). Referral still best rate, MyCareersFuture
  still lowest cost per hire.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/labs/lab-03-pivottables-pivotcharts-and-visuals/data/BrightPath_Recruitment_Metrics.xlsx
+++ b/labs/lab-03-pivottables-pivotcharts-and-visuals/data/BrightPath_Recruitment_Metrics.xlsx
@@ -4654,13 +4654,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>378</v>
+        <v>1735</v>
       </c>
       <c r="C2" t="n">
-        <v>17</v>
+        <v>88</v>
       </c>
       <c r="D2" s="9" t="n">
-        <v>14900</v>
+        <v>66500</v>
       </c>
     </row>
     <row r="3">
@@ -4670,13 +4670,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>270</v>
+        <v>1308</v>
       </c>
       <c r="C3" t="n">
-        <v>10</v>
+        <v>62</v>
       </c>
       <c r="D3" s="9" t="n">
-        <v>6200</v>
+        <v>27800</v>
       </c>
     </row>
     <row r="4">
@@ -4686,13 +4686,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>213</v>
+        <v>1035</v>
       </c>
       <c r="C4" t="n">
-        <v>7</v>
+        <v>47</v>
       </c>
       <c r="D4" s="9" t="n">
-        <v>1300</v>
+        <v>5900</v>
       </c>
     </row>
     <row r="5">
@@ -4702,13 +4702,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>149</v>
+        <v>620</v>
       </c>
       <c r="C5" t="n">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="D5" s="9" t="n">
-        <v>8500</v>
+        <v>34200</v>
       </c>
     </row>
     <row r="6">
@@ -4718,13 +4718,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>175</v>
+        <v>712</v>
       </c>
       <c r="C6" t="n">
-        <v>8</v>
+        <v>42</v>
       </c>
       <c r="D6" s="9" t="n">
-        <v>1600</v>
+        <v>6600</v>
       </c>
     </row>
     <row r="7">
@@ -4734,13 +4734,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>78</v>
+        <v>421</v>
       </c>
       <c r="C7" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>2400</v>
+        <v>13600</v>
       </c>
     </row>
     <row r="8">
@@ -4750,13 +4750,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>175</v>
+        <v>785</v>
       </c>
       <c r="C8" t="n">
-        <v>11</v>
+        <v>52</v>
       </c>
       <c r="D8" s="9" t="n">
-        <v>2200</v>
+        <v>9900</v>
       </c>
     </row>
   </sheetData>

</xml_diff>